<commit_message>
chore(proctor): actualizar template visual de exportacion xlsx
</commit_message>
<xml_diff>
--- a/app/templates/Template_Proctor.xlsx
+++ b/app/templates/Template_Proctor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE287EAC-D3DC-4240-B489-A1AF6DF790E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B8D959-2B5B-40D6-A8A8-211AA6506958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -113,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="339">
   <si>
     <t>:</t>
   </si>
@@ -1175,18 +1175,6 @@
   </si>
   <si>
     <t>Equipo utilizado</t>
-  </si>
-  <si>
-    <t>si o no</t>
-  </si>
-  <si>
-    <t>Húmedo o Seco</t>
-  </si>
-  <si>
-    <t>Manual o mecanico</t>
-  </si>
-  <si>
-    <t>se colocara si se realiza el ensayo</t>
   </si>
   <si>
     <t xml:space="preserve">* W Perdida de masa seca constante (adicional), para metodo B es &lt; 0.1% </t>
@@ -4993,22 +4981,22 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="102" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="104" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="101" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="107" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="108" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="102" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5019,35 +5007,60 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="109" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="110" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="101" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="102" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="104" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="78" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="98" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5123,136 +5136,46 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="98" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="78" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="98" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="106" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="111" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="102" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="107" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="108" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="104" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="109" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="110" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="98" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="113" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="2" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5281,6 +5204,10 @@
     <xf numFmtId="0" fontId="55" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -5299,6 +5226,9 @@
     <xf numFmtId="164" fontId="14" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5310,6 +5240,130 @@
     </xf>
     <xf numFmtId="0" fontId="55" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="113" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="2" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="54" fillId="3" borderId="98" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="55" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="55" fillId="3" borderId="98" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="84" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="85" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="87" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="53" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="53" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="53" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="53" fillId="3" borderId="1" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -5325,68 +5379,9 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="84" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="179" fontId="22" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="85" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="87" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="53" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="53" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="53" fillId="3" borderId="97" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="53" fillId="3" borderId="1" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="96" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="54" fillId="3" borderId="98" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="55" fillId="3" borderId="78" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="55" fillId="3" borderId="98" xfId="4" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="106" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5412,9 +5407,56 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="179" fontId="22" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="80" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="81" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="75" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="92" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="85" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="87" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="17" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="13" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="13" borderId="86" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="13" borderId="88" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="13" borderId="89" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="12" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="6" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5467,57 +5509,6 @@
     <xf numFmtId="0" fontId="46" fillId="11" borderId="79" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="80" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="81" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="83" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="75" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="92" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="85" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="87" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="17" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="13" borderId="84" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="13" borderId="86" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="13" borderId="88" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="13" borderId="89" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="12" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="9" borderId="69" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5607,9 +5598,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -7002,13 +6990,6 @@
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
-          <a:endParaRPr lang="es-PE" sz="1000" b="0">
-            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="es-PE" sz="1000" b="0">
               <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
@@ -7088,13 +7069,6 @@
             </a:rPr>
             <a:t>Aprobado:</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="es-PE" sz="1000" b="0">
-            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
@@ -10082,74 +10056,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="580"/>
-      <c r="B1" s="581"/>
-      <c r="C1" s="581"/>
-      <c r="D1" s="581"/>
-      <c r="E1" s="581"/>
-      <c r="F1" s="581"/>
-      <c r="G1" s="581"/>
-      <c r="H1" s="581"/>
-      <c r="I1" s="582"/>
+      <c r="A1" s="585"/>
+      <c r="B1" s="586"/>
+      <c r="C1" s="586"/>
+      <c r="D1" s="586"/>
+      <c r="E1" s="586"/>
+      <c r="F1" s="586"/>
+      <c r="G1" s="586"/>
+      <c r="H1" s="586"/>
+      <c r="I1" s="587"/>
     </row>
     <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="583"/>
-      <c r="B2" s="584"/>
-      <c r="C2" s="584"/>
-      <c r="D2" s="584"/>
-      <c r="E2" s="584"/>
-      <c r="F2" s="584"/>
-      <c r="G2" s="584"/>
-      <c r="H2" s="584"/>
-      <c r="I2" s="585"/>
+      <c r="A2" s="588"/>
+      <c r="B2" s="589"/>
+      <c r="C2" s="589"/>
+      <c r="D2" s="589"/>
+      <c r="E2" s="589"/>
+      <c r="F2" s="589"/>
+      <c r="G2" s="589"/>
+      <c r="H2" s="589"/>
+      <c r="I2" s="590"/>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="583"/>
-      <c r="B3" s="584"/>
-      <c r="C3" s="584"/>
-      <c r="D3" s="584"/>
-      <c r="E3" s="584"/>
-      <c r="F3" s="584"/>
-      <c r="G3" s="584"/>
-      <c r="H3" s="584"/>
-      <c r="I3" s="585"/>
+      <c r="A3" s="588"/>
+      <c r="B3" s="589"/>
+      <c r="C3" s="589"/>
+      <c r="D3" s="589"/>
+      <c r="E3" s="589"/>
+      <c r="F3" s="589"/>
+      <c r="G3" s="589"/>
+      <c r="H3" s="589"/>
+      <c r="I3" s="590"/>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="586"/>
-      <c r="B4" s="587"/>
-      <c r="C4" s="587"/>
-      <c r="D4" s="587"/>
-      <c r="E4" s="587"/>
-      <c r="F4" s="587"/>
-      <c r="G4" s="587"/>
-      <c r="H4" s="587"/>
-      <c r="I4" s="588"/>
+      <c r="A4" s="591"/>
+      <c r="B4" s="592"/>
+      <c r="C4" s="592"/>
+      <c r="D4" s="592"/>
+      <c r="E4" s="592"/>
+      <c r="F4" s="592"/>
+      <c r="G4" s="592"/>
+      <c r="H4" s="592"/>
+      <c r="I4" s="593"/>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="589" t="s">
+      <c r="A5" s="594" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="589"/>
-      <c r="C5" s="589"/>
-      <c r="D5" s="589"/>
-      <c r="E5" s="589"/>
-      <c r="F5" s="589"/>
-      <c r="G5" s="589"/>
-      <c r="H5" s="589"/>
-      <c r="I5" s="589"/>
+      <c r="B5" s="594"/>
+      <c r="C5" s="594"/>
+      <c r="D5" s="594"/>
+      <c r="E5" s="594"/>
+      <c r="F5" s="594"/>
+      <c r="G5" s="594"/>
+      <c r="H5" s="594"/>
+      <c r="I5" s="594"/>
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="590" t="s">
+      <c r="A6" s="595" t="s">
         <v>279</v>
       </c>
-      <c r="B6" s="590"/>
-      <c r="C6" s="590"/>
-      <c r="D6" s="590"/>
-      <c r="E6" s="590"/>
-      <c r="F6" s="590"/>
-      <c r="G6" s="590"/>
-      <c r="H6" s="590"/>
-      <c r="I6" s="590"/>
+      <c r="B6" s="595"/>
+      <c r="C6" s="595"/>
+      <c r="D6" s="595"/>
+      <c r="E6" s="595"/>
+      <c r="F6" s="595"/>
+      <c r="G6" s="595"/>
+      <c r="H6" s="595"/>
+      <c r="I6" s="595"/>
       <c r="L6"/>
     </row>
     <row r="7" spans="1:12" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -10166,68 +10140,68 @@
     <row r="8" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="473"/>
       <c r="B8" s="559" t="s">
-        <v>342</v>
-      </c>
-      <c r="C8" s="598" t="s">
+        <v>338</v>
+      </c>
+      <c r="C8" s="603" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="599"/>
+      <c r="D8" s="604"/>
       <c r="E8" s="562"/>
-      <c r="F8" s="600" t="s">
-        <v>341</v>
-      </c>
-      <c r="G8" s="599"/>
+      <c r="F8" s="605" t="s">
+        <v>337</v>
+      </c>
+      <c r="G8" s="604"/>
       <c r="H8" s="560" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="I8" s="474"/>
     </row>
     <row r="9" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="557"/>
-      <c r="C9" s="755"/>
-      <c r="D9" s="602"/>
+      <c r="C9" s="608"/>
+      <c r="D9" s="607"/>
       <c r="E9" s="561"/>
-      <c r="F9" s="601"/>
-      <c r="G9" s="602"/>
+      <c r="F9" s="606"/>
+      <c r="G9" s="607"/>
       <c r="H9" s="558"/>
       <c r="I9" s="474"/>
     </row>
     <row r="10" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="476"/>
-      <c r="B10" s="593"/>
-      <c r="C10" s="593"/>
-      <c r="D10" s="593"/>
+      <c r="B10" s="598"/>
+      <c r="C10" s="598"/>
+      <c r="D10" s="598"/>
       <c r="E10" s="475"/>
-      <c r="F10" s="593"/>
-      <c r="G10" s="593"/>
+      <c r="F10" s="598"/>
+      <c r="G10" s="598"/>
       <c r="H10" s="475"/>
       <c r="I10" s="477"/>
     </row>
     <row r="11" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="594" t="s">
+      <c r="A11" s="599" t="s">
         <v>292</v>
       </c>
-      <c r="B11" s="595"/>
-      <c r="C11" s="595"/>
-      <c r="D11" s="595"/>
-      <c r="E11" s="596"/>
-      <c r="F11" s="595"/>
-      <c r="G11" s="595"/>
-      <c r="H11" s="595"/>
-      <c r="I11" s="597"/>
+      <c r="B11" s="600"/>
+      <c r="C11" s="600"/>
+      <c r="D11" s="600"/>
+      <c r="E11" s="601"/>
+      <c r="F11" s="600"/>
+      <c r="G11" s="600"/>
+      <c r="H11" s="600"/>
+      <c r="I11" s="602"/>
     </row>
     <row r="12" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="605" t="s">
-        <v>331</v>
-      </c>
-      <c r="B12" s="606"/>
-      <c r="C12" s="607"/>
-      <c r="D12" s="606"/>
-      <c r="E12" s="607"/>
-      <c r="F12" s="606"/>
-      <c r="G12" s="607"/>
-      <c r="H12" s="606"/>
-      <c r="I12" s="608"/>
+      <c r="A12" s="577" t="s">
+        <v>327</v>
+      </c>
+      <c r="B12" s="578"/>
+      <c r="C12" s="579"/>
+      <c r="D12" s="578"/>
+      <c r="E12" s="579"/>
+      <c r="F12" s="578"/>
+      <c r="G12" s="579"/>
+      <c r="H12" s="578"/>
+      <c r="I12" s="580"/>
     </row>
     <row r="13" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="478"/>
@@ -10256,120 +10230,120 @@
       <c r="I14" s="488"/>
     </row>
     <row r="15" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="565" t="s">
+      <c r="A15" s="581" t="s">
         <v>253</v>
       </c>
-      <c r="B15" s="565"/>
+      <c r="B15" s="581"/>
       <c r="C15" s="489" t="s">
         <v>287</v>
       </c>
-      <c r="D15" s="591"/>
-      <c r="E15" s="592"/>
+      <c r="D15" s="596"/>
+      <c r="E15" s="597"/>
       <c r="F15" s="490"/>
       <c r="G15" s="491"/>
       <c r="H15" s="491"/>
       <c r="I15" s="490"/>
     </row>
     <row r="16" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="566" t="s">
+      <c r="A16" s="576" t="s">
         <v>254</v>
       </c>
-      <c r="B16" s="566"/>
+      <c r="B16" s="576"/>
       <c r="C16" s="492" t="s">
         <v>287</v>
       </c>
-      <c r="D16" s="563"/>
-      <c r="E16" s="564"/>
+      <c r="D16" s="566"/>
+      <c r="E16" s="567"/>
       <c r="F16" s="493"/>
       <c r="G16" s="494"/>
       <c r="H16" s="494"/>
       <c r="I16" s="493"/>
     </row>
     <row r="17" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="566" t="s">
+      <c r="A17" s="576" t="s">
         <v>255</v>
       </c>
-      <c r="B17" s="566"/>
+      <c r="B17" s="576"/>
       <c r="C17" s="492" t="s">
         <v>287</v>
       </c>
-      <c r="D17" s="563"/>
-      <c r="E17" s="564"/>
+      <c r="D17" s="566"/>
+      <c r="E17" s="567"/>
       <c r="F17" s="493"/>
       <c r="G17" s="494"/>
       <c r="H17" s="494"/>
       <c r="I17" s="493"/>
     </row>
     <row r="18" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="566" t="s">
+      <c r="A18" s="576" t="s">
         <v>303</v>
       </c>
-      <c r="B18" s="566"/>
+      <c r="B18" s="576"/>
       <c r="C18" s="494" t="s">
         <v>288</v>
       </c>
-      <c r="D18" s="563"/>
-      <c r="E18" s="564"/>
+      <c r="D18" s="566"/>
+      <c r="E18" s="567"/>
       <c r="F18" s="495"/>
       <c r="G18" s="496"/>
       <c r="H18" s="496"/>
       <c r="I18" s="495"/>
     </row>
     <row r="19" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="566" t="s">
+      <c r="A19" s="576" t="s">
         <v>302</v>
       </c>
-      <c r="B19" s="566"/>
+      <c r="B19" s="576"/>
       <c r="C19" s="494" t="s">
         <v>288</v>
       </c>
-      <c r="D19" s="563"/>
-      <c r="E19" s="564"/>
+      <c r="D19" s="566"/>
+      <c r="E19" s="567"/>
       <c r="F19" s="493"/>
       <c r="G19" s="494"/>
       <c r="H19" s="497"/>
       <c r="I19" s="498"/>
     </row>
     <row r="20" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="609" t="s">
+      <c r="A20" s="582" t="s">
         <v>301</v>
       </c>
-      <c r="B20" s="610"/>
+      <c r="B20" s="583"/>
       <c r="C20" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D20" s="563"/>
-      <c r="E20" s="564"/>
+      <c r="D20" s="566"/>
+      <c r="E20" s="567"/>
       <c r="F20" s="493"/>
       <c r="G20" s="494"/>
       <c r="H20" s="497"/>
       <c r="I20" s="498"/>
     </row>
     <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="566" t="s">
+      <c r="A21" s="576" t="s">
         <v>300</v>
       </c>
-      <c r="B21" s="566"/>
+      <c r="B21" s="576"/>
       <c r="C21" s="494" t="s">
         <v>290</v>
       </c>
-      <c r="D21" s="563"/>
-      <c r="E21" s="564"/>
+      <c r="D21" s="566"/>
+      <c r="E21" s="567"/>
       <c r="F21" s="493"/>
       <c r="G21" s="494"/>
       <c r="H21" s="494"/>
       <c r="I21" s="493"/>
     </row>
     <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="572" t="s">
+      <c r="A22" s="584" t="s">
         <v>299</v>
       </c>
-      <c r="B22" s="572"/>
+      <c r="B22" s="584"/>
       <c r="C22" s="500" t="s">
         <v>289</v>
       </c>
-      <c r="D22" s="563"/>
-      <c r="E22" s="564"/>
+      <c r="D22" s="566"/>
+      <c r="E22" s="567"/>
       <c r="F22" s="501"/>
       <c r="G22" s="502"/>
       <c r="H22" s="502"/>
@@ -10389,148 +10363,148 @@
       <c r="I23" s="503"/>
     </row>
     <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="565" t="s">
+      <c r="A24" s="581" t="s">
         <v>256</v>
       </c>
-      <c r="B24" s="565"/>
+      <c r="B24" s="581"/>
       <c r="C24" s="504"/>
-      <c r="D24" s="567"/>
-      <c r="E24" s="568"/>
+      <c r="D24" s="614"/>
+      <c r="E24" s="615"/>
       <c r="F24" s="505"/>
       <c r="G24" s="506"/>
       <c r="H24" s="506"/>
       <c r="I24" s="505"/>
     </row>
     <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="566" t="s">
+      <c r="A25" s="576" t="s">
         <v>304</v>
       </c>
-      <c r="B25" s="566"/>
+      <c r="B25" s="576"/>
       <c r="C25" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D25" s="569"/>
-      <c r="E25" s="570"/>
+      <c r="D25" s="568"/>
+      <c r="E25" s="569"/>
       <c r="F25" s="507"/>
       <c r="G25" s="508"/>
       <c r="H25" s="508"/>
       <c r="I25" s="507"/>
     </row>
     <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="566" t="s">
+      <c r="A26" s="576" t="s">
         <v>305</v>
       </c>
-      <c r="B26" s="566"/>
+      <c r="B26" s="576"/>
       <c r="C26" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D26" s="569"/>
-      <c r="E26" s="570"/>
+      <c r="D26" s="568"/>
+      <c r="E26" s="569"/>
       <c r="F26" s="507"/>
       <c r="G26" s="508"/>
       <c r="H26" s="508"/>
       <c r="I26" s="507"/>
     </row>
     <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="566" t="s">
+      <c r="A27" s="576" t="s">
         <v>298</v>
       </c>
-      <c r="B27" s="566"/>
+      <c r="B27" s="576"/>
       <c r="C27" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D27" s="569"/>
-      <c r="E27" s="570"/>
+      <c r="D27" s="568"/>
+      <c r="E27" s="569"/>
       <c r="F27" s="507"/>
       <c r="G27" s="508"/>
       <c r="H27" s="508"/>
       <c r="I27" s="507"/>
     </row>
     <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="566" t="s">
+      <c r="A28" s="576" t="s">
         <v>306</v>
       </c>
-      <c r="B28" s="566"/>
+      <c r="B28" s="576"/>
       <c r="C28" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D28" s="569"/>
-      <c r="E28" s="570"/>
+      <c r="D28" s="568"/>
+      <c r="E28" s="569"/>
       <c r="F28" s="507"/>
       <c r="G28" s="508"/>
       <c r="H28" s="508"/>
       <c r="I28" s="507"/>
     </row>
     <row r="29" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="566" t="s">
+      <c r="A29" s="576" t="s">
         <v>307</v>
       </c>
-      <c r="B29" s="566"/>
+      <c r="B29" s="576"/>
       <c r="C29" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D29" s="569"/>
-      <c r="E29" s="570"/>
+      <c r="D29" s="568"/>
+      <c r="E29" s="569"/>
       <c r="F29" s="509"/>
       <c r="G29" s="510"/>
       <c r="H29" s="510"/>
       <c r="I29" s="509"/>
     </row>
     <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="566" t="s">
+      <c r="A30" s="576" t="s">
         <v>308</v>
       </c>
-      <c r="B30" s="566"/>
+      <c r="B30" s="576"/>
       <c r="C30" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D30" s="569"/>
-      <c r="E30" s="570"/>
+      <c r="D30" s="568"/>
+      <c r="E30" s="569"/>
       <c r="F30" s="509"/>
       <c r="G30" s="510"/>
       <c r="H30" s="510"/>
       <c r="I30" s="509"/>
     </row>
     <row r="31" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="566" t="s">
+      <c r="A31" s="576" t="s">
         <v>309</v>
       </c>
-      <c r="B31" s="566"/>
+      <c r="B31" s="576"/>
       <c r="C31" s="499" t="s">
         <v>288</v>
       </c>
-      <c r="D31" s="569"/>
-      <c r="E31" s="570"/>
+      <c r="D31" s="568"/>
+      <c r="E31" s="569"/>
       <c r="F31" s="509"/>
       <c r="G31" s="510"/>
       <c r="H31" s="510"/>
       <c r="I31" s="509"/>
     </row>
     <row r="32" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="566" t="s">
+      <c r="A32" s="576" t="s">
         <v>310</v>
       </c>
-      <c r="B32" s="566"/>
+      <c r="B32" s="576"/>
       <c r="C32" s="494" t="s">
         <v>291</v>
       </c>
-      <c r="D32" s="569"/>
-      <c r="E32" s="570"/>
+      <c r="D32" s="568"/>
+      <c r="E32" s="569"/>
       <c r="F32" s="511"/>
       <c r="G32" s="512"/>
       <c r="H32" s="512"/>
       <c r="I32" s="511"/>
     </row>
     <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="572" t="s">
+      <c r="A33" s="584" t="s">
         <v>323</v>
       </c>
-      <c r="B33" s="572"/>
+      <c r="B33" s="584"/>
       <c r="C33" s="500" t="s">
         <v>289</v>
       </c>
-      <c r="D33" s="611"/>
-      <c r="E33" s="612"/>
+      <c r="D33" s="570"/>
+      <c r="E33" s="571"/>
       <c r="F33" s="501"/>
       <c r="G33" s="502"/>
       <c r="H33" s="502"/>
@@ -10543,7 +10517,7 @@
       <c r="B34" s="514"/>
       <c r="C34" s="514"/>
       <c r="D34" s="515" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E34" s="516"/>
       <c r="F34" s="516"/>
@@ -10556,19 +10530,19 @@
         <v>316</v>
       </c>
       <c r="B35" s="520"/>
-      <c r="C35" s="613"/>
-      <c r="D35" s="614"/>
+      <c r="C35" s="572"/>
+      <c r="D35" s="573"/>
       <c r="E35" s="521"/>
-      <c r="F35" s="578" t="s">
+      <c r="F35" s="612" t="s">
         <v>311</v>
       </c>
-      <c r="G35" s="578" t="s">
+      <c r="G35" s="612" t="s">
         <v>312</v>
       </c>
-      <c r="H35" s="578" t="s">
+      <c r="H35" s="612" t="s">
         <v>280</v>
       </c>
-      <c r="I35" s="578" t="s">
+      <c r="I35" s="612" t="s">
         <v>257</v>
       </c>
     </row>
@@ -10577,21 +10551,21 @@
         <v>317</v>
       </c>
       <c r="B36" s="523"/>
-      <c r="C36" s="613"/>
-      <c r="D36" s="614"/>
+      <c r="C36" s="572"/>
+      <c r="D36" s="573"/>
       <c r="E36" s="521"/>
-      <c r="F36" s="579"/>
-      <c r="G36" s="579"/>
-      <c r="H36" s="579"/>
-      <c r="I36" s="579"/>
+      <c r="F36" s="613"/>
+      <c r="G36" s="613"/>
+      <c r="H36" s="613"/>
+      <c r="I36" s="613"/>
     </row>
     <row r="37" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="522" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B37" s="523"/>
-      <c r="C37" s="613"/>
-      <c r="D37" s="614"/>
+      <c r="C37" s="572"/>
+      <c r="D37" s="573"/>
       <c r="E37" s="524"/>
       <c r="F37" s="525" t="s">
         <v>293</v>
@@ -10605,8 +10579,8 @@
         <v>318</v>
       </c>
       <c r="B38" s="530"/>
-      <c r="C38" s="613"/>
-      <c r="D38" s="614"/>
+      <c r="C38" s="572"/>
+      <c r="D38" s="573"/>
       <c r="E38" s="521"/>
       <c r="F38" s="525" t="s">
         <v>294</v>
@@ -10620,11 +10594,11 @@
         <v>319</v>
       </c>
       <c r="B39" s="523"/>
-      <c r="C39" s="613"/>
-      <c r="D39" s="614"/>
+      <c r="C39" s="572"/>
+      <c r="D39" s="573"/>
       <c r="E39" s="521"/>
       <c r="F39" s="525" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="G39" s="526"/>
       <c r="H39" s="527"/>
@@ -10639,7 +10613,7 @@
       <c r="D40" s="531"/>
       <c r="E40" s="531"/>
       <c r="F40" s="525" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G40" s="526"/>
       <c r="H40" s="528"/>
@@ -10650,8 +10624,8 @@
         <v>295</v>
       </c>
       <c r="B41" s="533"/>
-      <c r="C41" s="577"/>
-      <c r="D41" s="577"/>
+      <c r="C41" s="565"/>
+      <c r="D41" s="565"/>
       <c r="E41" s="531"/>
       <c r="F41" s="525" t="s">
         <v>297</v>
@@ -10665,68 +10639,60 @@
         <v>314</v>
       </c>
       <c r="B42" s="536"/>
-      <c r="C42" s="577"/>
-      <c r="D42" s="577"/>
+      <c r="C42" s="565"/>
+      <c r="D42" s="565"/>
       <c r="E42" s="537"/>
-      <c r="J42" s="538" t="s">
-        <v>327</v>
-      </c>
+      <c r="J42" s="538"/>
     </row>
     <row r="43" spans="1:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="539" t="s">
         <v>315</v>
       </c>
       <c r="B43" s="540"/>
-      <c r="C43" s="577"/>
-      <c r="D43" s="577"/>
+      <c r="C43" s="565"/>
+      <c r="D43" s="565"/>
       <c r="E43" s="537"/>
-      <c r="F43" s="603" t="s">
+      <c r="F43" s="574" t="s">
         <v>325</v>
       </c>
-      <c r="G43" s="604"/>
-      <c r="H43" s="573" t="s">
+      <c r="G43" s="575"/>
+      <c r="H43" s="563" t="s">
         <v>281</v>
       </c>
-      <c r="I43" s="574"/>
-      <c r="J43" s="538" t="s">
-        <v>328</v>
-      </c>
+      <c r="I43" s="564"/>
+      <c r="J43" s="538"/>
     </row>
     <row r="44" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="532" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="B44" s="536"/>
-      <c r="C44" s="577"/>
-      <c r="D44" s="577"/>
+      <c r="C44" s="565"/>
+      <c r="D44" s="565"/>
       <c r="E44" s="537"/>
       <c r="F44" s="541" t="s">
         <v>296</v>
       </c>
       <c r="G44" s="542"/>
-      <c r="H44" s="573"/>
-      <c r="I44" s="574"/>
-      <c r="J44" s="538" t="s">
-        <v>329</v>
-      </c>
+      <c r="H44" s="563"/>
+      <c r="I44" s="564"/>
+      <c r="J44" s="538"/>
     </row>
     <row r="45" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="575" t="s">
-        <v>334</v>
-      </c>
-      <c r="B45" s="576"/>
-      <c r="C45" s="577"/>
-      <c r="D45" s="577"/>
+      <c r="A45" s="610" t="s">
+        <v>330</v>
+      </c>
+      <c r="B45" s="611"/>
+      <c r="C45" s="565"/>
+      <c r="D45" s="565"/>
       <c r="E45" s="537"/>
       <c r="F45" s="541" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="G45" s="542"/>
-      <c r="H45" s="573"/>
-      <c r="I45" s="574"/>
-      <c r="J45" s="538" t="s">
-        <v>326</v>
-      </c>
+      <c r="H45" s="563"/>
+      <c r="I45" s="564"/>
+      <c r="J45" s="538"/>
     </row>
     <row r="46" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="543" t="s">
@@ -10739,8 +10705,8 @@
         <v>320</v>
       </c>
       <c r="G46" s="542"/>
-      <c r="H46" s="573"/>
-      <c r="I46" s="574"/>
+      <c r="H46" s="563"/>
+      <c r="I46" s="564"/>
     </row>
     <row r="47" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="546"/>
@@ -10748,11 +10714,11 @@
       <c r="C47" s="547"/>
       <c r="D47" s="548"/>
       <c r="F47" s="541" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="G47" s="542"/>
-      <c r="H47" s="573"/>
-      <c r="I47" s="574"/>
+      <c r="H47" s="563"/>
+      <c r="I47" s="564"/>
     </row>
     <row r="48" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="546"/>
@@ -10763,8 +10729,8 @@
         <v>282</v>
       </c>
       <c r="G48" s="549"/>
-      <c r="H48" s="573"/>
-      <c r="I48" s="574"/>
+      <c r="H48" s="563"/>
+      <c r="I48" s="564"/>
     </row>
     <row r="49" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="550"/>
@@ -10775,8 +10741,8 @@
         <v>283</v>
       </c>
       <c r="G49" s="542"/>
-      <c r="H49" s="577"/>
-      <c r="I49" s="577"/>
+      <c r="H49" s="565"/>
+      <c r="I49" s="565"/>
     </row>
     <row r="50" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E50" s="553"/>
@@ -10802,7 +10768,7 @@
     </row>
     <row r="54" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="554" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B54" s="44"/>
       <c r="C54" s="44"/>
@@ -10817,17 +10783,17 @@
     </row>
     <row r="55" spans="1:9" ht="0.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="571" t="s">
+      <c r="A56" s="609" t="s">
         <v>278</v>
       </c>
-      <c r="B56" s="571"/>
-      <c r="C56" s="571"/>
-      <c r="D56" s="571"/>
-      <c r="E56" s="571"/>
-      <c r="F56" s="571"/>
-      <c r="G56" s="571"/>
-      <c r="H56" s="571"/>
-      <c r="I56" s="571"/>
+      <c r="B56" s="609"/>
+      <c r="C56" s="609"/>
+      <c r="D56" s="609"/>
+      <c r="E56" s="609"/>
+      <c r="F56" s="609"/>
+      <c r="G56" s="609"/>
+      <c r="H56" s="609"/>
+      <c r="I56" s="609"/>
     </row>
     <row r="57" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -10837,53 +10803,13 @@
     <protectedRange sqref="B9:C10" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="71">
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A1:I4"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="A56:I56"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A29:B29"/>
@@ -10900,14 +10826,54 @@
     <mergeCell ref="H35:H36"/>
     <mergeCell ref="I35:I36"/>
     <mergeCell ref="D27:E27"/>
+    <mergeCell ref="A1:I4"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
     <mergeCell ref="D21:E21"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -11117,19 +11083,19 @@
       <c r="Z6" s="51"/>
     </row>
     <row r="7" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="644" t="s">
+      <c r="A7" s="623" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="644"/>
-      <c r="C7" s="644"/>
-      <c r="D7" s="644"/>
-      <c r="E7" s="644"/>
-      <c r="F7" s="644"/>
-      <c r="G7" s="644"/>
-      <c r="H7" s="644"/>
-      <c r="I7" s="644"/>
-      <c r="J7" s="644"/>
-      <c r="K7" s="644"/>
+      <c r="B7" s="623"/>
+      <c r="C7" s="623"/>
+      <c r="D7" s="623"/>
+      <c r="E7" s="623"/>
+      <c r="F7" s="623"/>
+      <c r="G7" s="623"/>
+      <c r="H7" s="623"/>
+      <c r="I7" s="623"/>
+      <c r="J7" s="623"/>
+      <c r="K7" s="623"/>
       <c r="N7" s="469" t="s">
         <v>73</v>
       </c>
@@ -11154,20 +11120,20 @@
       <c r="Z7" s="51"/>
     </row>
     <row r="8" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="645">
+      <c r="A8" s="624">
         <f>+K12</f>
         <v>1</v>
       </c>
-      <c r="B8" s="645"/>
-      <c r="C8" s="645"/>
-      <c r="D8" s="645"/>
-      <c r="E8" s="645"/>
-      <c r="F8" s="645"/>
-      <c r="G8" s="645"/>
-      <c r="H8" s="645"/>
-      <c r="I8" s="645"/>
-      <c r="J8" s="645"/>
-      <c r="K8" s="645"/>
+      <c r="B8" s="624"/>
+      <c r="C8" s="624"/>
+      <c r="D8" s="624"/>
+      <c r="E8" s="624"/>
+      <c r="F8" s="624"/>
+      <c r="G8" s="624"/>
+      <c r="H8" s="624"/>
+      <c r="I8" s="624"/>
+      <c r="J8" s="624"/>
+      <c r="K8" s="624"/>
       <c r="N8" s="343" t="s">
         <v>74</v>
       </c>
@@ -11222,14 +11188,14 @@
       <c r="B10" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="638" t="s">
+      <c r="C10" s="647" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="638"/>
-      <c r="E10" s="638"/>
-      <c r="F10" s="638"/>
-      <c r="G10" s="638"/>
-      <c r="H10" s="638"/>
+      <c r="D10" s="647"/>
+      <c r="E10" s="647"/>
+      <c r="F10" s="647"/>
+      <c r="G10" s="647"/>
+      <c r="H10" s="647"/>
       <c r="I10" s="36" t="s">
         <v>38</v>
       </c>
@@ -11272,14 +11238,14 @@
       <c r="B11" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="638" t="s">
+      <c r="C11" s="647" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="638"/>
-      <c r="E11" s="638"/>
-      <c r="F11" s="638"/>
-      <c r="G11" s="638"/>
-      <c r="H11" s="638"/>
+      <c r="D11" s="647"/>
+      <c r="E11" s="647"/>
+      <c r="F11" s="647"/>
+      <c r="G11" s="647"/>
+      <c r="H11" s="647"/>
       <c r="I11" s="39" t="s">
         <v>21</v>
       </c>
@@ -11321,14 +11287,14 @@
       <c r="B12" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="638" t="s">
+      <c r="C12" s="647" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="638"/>
-      <c r="E12" s="638"/>
-      <c r="F12" s="638"/>
-      <c r="G12" s="638"/>
-      <c r="H12" s="638"/>
+      <c r="D12" s="647"/>
+      <c r="E12" s="647"/>
+      <c r="F12" s="647"/>
+      <c r="G12" s="647"/>
+      <c r="H12" s="647"/>
       <c r="I12" s="39" t="s">
         <v>22</v>
       </c>
@@ -11408,19 +11374,19 @@
       <c r="Z13" s="51"/>
     </row>
     <row r="14" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="594" t="s">
+      <c r="A14" s="599" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="595"/>
-      <c r="C14" s="595"/>
-      <c r="D14" s="595"/>
-      <c r="E14" s="595"/>
-      <c r="F14" s="595"/>
-      <c r="G14" s="595"/>
-      <c r="H14" s="595"/>
-      <c r="I14" s="595"/>
-      <c r="J14" s="595"/>
-      <c r="K14" s="597"/>
+      <c r="B14" s="600"/>
+      <c r="C14" s="600"/>
+      <c r="D14" s="600"/>
+      <c r="E14" s="600"/>
+      <c r="F14" s="600"/>
+      <c r="G14" s="600"/>
+      <c r="H14" s="600"/>
+      <c r="I14" s="600"/>
+      <c r="J14" s="600"/>
+      <c r="K14" s="602"/>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
       <c r="N14" s="343" t="s">
@@ -11443,19 +11409,19 @@
       <c r="Z14" s="51"/>
     </row>
     <row r="15" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="605" t="s">
+      <c r="A15" s="577" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="606"/>
-      <c r="C15" s="606"/>
-      <c r="D15" s="606"/>
-      <c r="E15" s="606"/>
-      <c r="F15" s="606"/>
-      <c r="G15" s="606"/>
-      <c r="H15" s="606"/>
-      <c r="I15" s="606"/>
-      <c r="J15" s="606"/>
-      <c r="K15" s="608"/>
+      <c r="B15" s="578"/>
+      <c r="C15" s="578"/>
+      <c r="D15" s="578"/>
+      <c r="E15" s="578"/>
+      <c r="F15" s="578"/>
+      <c r="G15" s="578"/>
+      <c r="H15" s="578"/>
+      <c r="I15" s="578"/>
+      <c r="J15" s="578"/>
+      <c r="K15" s="580"/>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
       <c r="N15" s="38"/>
@@ -11502,30 +11468,30 @@
       <c r="S16" s="366" t="s">
         <v>45</v>
       </c>
-      <c r="T16" s="618" t="s">
+      <c r="T16" s="651" t="s">
         <v>99</v>
       </c>
-      <c r="U16" s="619"/>
-      <c r="V16" s="620"/>
+      <c r="U16" s="652"/>
+      <c r="V16" s="653"/>
       <c r="W16" s="51"/>
       <c r="X16" s="51"/>
       <c r="Y16" s="51"/>
       <c r="Z16" s="51"/>
     </row>
     <row r="17" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="635" t="s">
+      <c r="A17" s="644" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="636"/>
-      <c r="C17" s="636"/>
-      <c r="D17" s="636"/>
-      <c r="E17" s="636"/>
-      <c r="F17" s="636"/>
-      <c r="G17" s="636"/>
-      <c r="H17" s="636"/>
-      <c r="I17" s="636"/>
-      <c r="J17" s="636"/>
-      <c r="K17" s="637"/>
+      <c r="B17" s="645"/>
+      <c r="C17" s="645"/>
+      <c r="D17" s="645"/>
+      <c r="E17" s="645"/>
+      <c r="F17" s="645"/>
+      <c r="G17" s="645"/>
+      <c r="H17" s="645"/>
+      <c r="I17" s="645"/>
+      <c r="J17" s="645"/>
+      <c r="K17" s="646"/>
       <c r="M17" s="15"/>
       <c r="N17" s="367" t="s">
         <v>46</v>
@@ -11545,11 +11511,11 @@
       <c r="S17" s="368" t="s">
         <v>48</v>
       </c>
-      <c r="T17" s="615" t="s">
+      <c r="T17" s="648" t="s">
         <v>276</v>
       </c>
-      <c r="U17" s="616"/>
-      <c r="V17" s="617"/>
+      <c r="U17" s="649"/>
+      <c r="V17" s="650"/>
       <c r="W17" s="51"/>
       <c r="X17" s="51"/>
       <c r="Y17" s="51"/>
@@ -11809,21 +11775,21 @@
       <c r="Z22" s="51"/>
     </row>
     <row r="23" spans="1:26" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="648" t="s">
+      <c r="A23" s="627" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="649"/>
-      <c r="C23" s="650"/>
-      <c r="D23" s="623" t="s">
+      <c r="B23" s="628"/>
+      <c r="C23" s="629"/>
+      <c r="D23" s="655" t="s">
         <v>57</v>
       </c>
       <c r="E23" s="313"/>
-      <c r="F23" s="651" t="s">
+      <c r="F23" s="631" t="s">
         <v>98</v>
       </c>
-      <c r="G23" s="652"/>
-      <c r="H23" s="653"/>
-      <c r="I23" s="628" t="s">
+      <c r="G23" s="632"/>
+      <c r="H23" s="633"/>
+      <c r="I23" s="637" t="s">
         <v>50</v>
       </c>
       <c r="J23" s="307"/>
@@ -11867,16 +11833,16 @@
       <c r="A24" s="314" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="647" t="s">
+      <c r="B24" s="626" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="647"/>
-      <c r="D24" s="624"/>
+      <c r="C24" s="626"/>
+      <c r="D24" s="656"/>
       <c r="E24" s="313"/>
-      <c r="F24" s="654"/>
-      <c r="G24" s="655"/>
-      <c r="H24" s="656"/>
-      <c r="I24" s="657"/>
+      <c r="F24" s="634"/>
+      <c r="G24" s="635"/>
+      <c r="H24" s="636"/>
+      <c r="I24" s="638"/>
       <c r="J24" s="307"/>
       <c r="K24" s="308"/>
       <c r="L24" s="15"/>
@@ -11914,10 +11880,10 @@
       <c r="A25" s="315" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="646">
+      <c r="B25" s="625">
         <v>76.2</v>
       </c>
-      <c r="C25" s="646"/>
+      <c r="C25" s="625"/>
       <c r="D25" s="316">
         <f>+S18</f>
         <v>100</v>
@@ -11968,21 +11934,21 @@
       <c r="A26" s="317" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="622">
+      <c r="B26" s="630">
         <v>50.6</v>
       </c>
-      <c r="C26" s="622"/>
+      <c r="C26" s="630"/>
       <c r="D26" s="318">
         <f>+S20</f>
         <v>96.737365729020368</v>
       </c>
       <c r="E26" s="313"/>
-      <c r="F26" s="648" t="s">
+      <c r="F26" s="627" t="s">
         <v>64</v>
       </c>
-      <c r="G26" s="649"/>
-      <c r="H26" s="649"/>
-      <c r="I26" s="650"/>
+      <c r="G26" s="628"/>
+      <c r="H26" s="628"/>
+      <c r="I26" s="629"/>
       <c r="J26" s="319"/>
       <c r="K26" s="320"/>
       <c r="L26" s="15"/>
@@ -12020,19 +11986,19 @@
       <c r="A27" s="321" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="622">
+      <c r="B27" s="630">
         <v>38.1</v>
       </c>
-      <c r="C27" s="622"/>
+      <c r="C27" s="630"/>
       <c r="D27" s="318">
         <f>+S21</f>
         <v>90.324022891039832</v>
       </c>
       <c r="E27" s="313"/>
-      <c r="F27" s="658"/>
-      <c r="G27" s="659"/>
-      <c r="H27" s="659"/>
-      <c r="I27" s="660"/>
+      <c r="F27" s="639"/>
+      <c r="G27" s="640"/>
+      <c r="H27" s="640"/>
+      <c r="I27" s="641"/>
       <c r="J27" s="319"/>
       <c r="K27" s="320"/>
       <c r="L27" s="15"/>
@@ -12074,19 +12040,19 @@
       <c r="A28" s="317" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="622">
+      <c r="B28" s="630">
         <v>25.4</v>
       </c>
-      <c r="C28" s="622"/>
+      <c r="C28" s="630"/>
       <c r="D28" s="318">
         <f>+S22</f>
         <v>84.873241107276272</v>
       </c>
       <c r="E28" s="313"/>
-      <c r="F28" s="631" t="s">
+      <c r="F28" s="642" t="s">
         <v>58</v>
       </c>
-      <c r="G28" s="633">
+      <c r="G28" s="643">
         <f>R27</f>
         <v>45.788805497693524</v>
       </c>
@@ -12134,17 +12100,17 @@
       <c r="A29" s="317" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="622">
+      <c r="B29" s="630">
         <v>19.05</v>
       </c>
-      <c r="C29" s="622"/>
+      <c r="C29" s="630"/>
       <c r="D29" s="318">
         <f>+S23</f>
         <v>73.456819301447041</v>
       </c>
       <c r="E29" s="313"/>
-      <c r="F29" s="632"/>
-      <c r="G29" s="634"/>
+      <c r="F29" s="618"/>
+      <c r="G29" s="621"/>
       <c r="H29" s="324" t="s">
         <v>60</v>
       </c>
@@ -12193,19 +12159,19 @@
       <c r="A30" s="317" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="622">
+      <c r="B30" s="630">
         <v>9.5250000000000004</v>
       </c>
-      <c r="C30" s="622"/>
+      <c r="C30" s="630"/>
       <c r="D30" s="318">
         <f>+S25</f>
         <v>62.661585152699679</v>
       </c>
       <c r="E30" s="313"/>
-      <c r="F30" s="639" t="s">
+      <c r="F30" s="616" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="641">
+      <c r="G30" s="619">
         <f>100-(G28+G33)</f>
         <v>40.754382185876274</v>
       </c>
@@ -12253,17 +12219,17 @@
       <c r="A31" s="317" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="622">
+      <c r="B31" s="630">
         <v>4.76</v>
       </c>
-      <c r="C31" s="622"/>
+      <c r="C31" s="630"/>
       <c r="D31" s="318">
         <f>+S27</f>
         <v>54.211194502306476</v>
       </c>
       <c r="E31" s="313"/>
-      <c r="F31" s="640"/>
-      <c r="G31" s="642"/>
+      <c r="F31" s="617"/>
+      <c r="G31" s="620"/>
       <c r="H31" s="324" t="s">
         <v>62</v>
       </c>
@@ -12311,17 +12277,17 @@
       <c r="A32" s="317">
         <v>8</v>
       </c>
-      <c r="B32" s="622">
+      <c r="B32" s="630">
         <v>2.36</v>
       </c>
-      <c r="C32" s="622"/>
+      <c r="C32" s="630"/>
       <c r="D32" s="318">
         <f>+S28</f>
         <v>49.032616067382399</v>
       </c>
       <c r="E32" s="313"/>
-      <c r="F32" s="632"/>
-      <c r="G32" s="634"/>
+      <c r="F32" s="618"/>
+      <c r="G32" s="621"/>
       <c r="H32" s="324" t="s">
         <v>60</v>
       </c>
@@ -12373,10 +12339,10 @@
       <c r="A33" s="317">
         <v>16</v>
       </c>
-      <c r="B33" s="622">
+      <c r="B33" s="630">
         <v>1.19</v>
       </c>
-      <c r="C33" s="622"/>
+      <c r="C33" s="630"/>
       <c r="D33" s="318">
         <f t="shared" ref="D33:D38" si="4">+S30</f>
         <v>40.351707913359583</v>
@@ -12431,10 +12397,10 @@
       <c r="A34" s="317">
         <v>30</v>
       </c>
-      <c r="B34" s="622">
+      <c r="B34" s="630">
         <v>0.6</v>
       </c>
-      <c r="C34" s="622"/>
+      <c r="C34" s="630"/>
       <c r="D34" s="318">
         <f t="shared" si="4"/>
         <v>31.408593256302638</v>
@@ -12481,25 +12447,25 @@
       <c r="A35" s="317">
         <v>40</v>
       </c>
-      <c r="B35" s="622">
+      <c r="B35" s="630">
         <v>0.42</v>
       </c>
-      <c r="C35" s="622"/>
+      <c r="C35" s="630"/>
       <c r="D35" s="318">
         <f t="shared" si="4"/>
         <v>27.175831135894526</v>
       </c>
       <c r="E35" s="313"/>
-      <c r="F35" s="625" t="str">
+      <c r="F35" s="657" t="str">
         <f>IF(O3="No","","Clasificacion SUCS")</f>
         <v/>
       </c>
-      <c r="G35" s="625"/>
-      <c r="H35" s="628" t="str">
+      <c r="G35" s="657"/>
+      <c r="H35" s="637" t="str">
         <f>IF(O3="No","",'Sucs '!G4)</f>
         <v/>
       </c>
-      <c r="I35" s="628"/>
+      <c r="I35" s="637"/>
       <c r="J35" s="319"/>
       <c r="K35" s="320"/>
       <c r="L35" s="15"/>
@@ -12541,19 +12507,19 @@
       <c r="A36" s="317">
         <v>50</v>
       </c>
-      <c r="B36" s="622">
+      <c r="B36" s="630">
         <v>0.3</v>
       </c>
-      <c r="C36" s="622"/>
+      <c r="C36" s="630"/>
       <c r="D36" s="318">
         <f t="shared" si="4"/>
         <v>23.785875632381845</v>
       </c>
       <c r="E36" s="313"/>
-      <c r="F36" s="626"/>
-      <c r="G36" s="626"/>
-      <c r="H36" s="629"/>
-      <c r="I36" s="629"/>
+      <c r="F36" s="658"/>
+      <c r="G36" s="658"/>
+      <c r="H36" s="660"/>
+      <c r="I36" s="660"/>
       <c r="J36" s="319"/>
       <c r="K36" s="320"/>
       <c r="L36" s="15"/>
@@ -12592,25 +12558,25 @@
       <c r="A37" s="317">
         <v>100</v>
       </c>
-      <c r="B37" s="622">
+      <c r="B37" s="630">
         <v>0.14899999999999999</v>
       </c>
-      <c r="C37" s="622"/>
+      <c r="C37" s="630"/>
       <c r="D37" s="318">
         <f t="shared" si="4"/>
         <v>17.820677688355374</v>
       </c>
       <c r="E37" s="313"/>
-      <c r="F37" s="626" t="str">
+      <c r="F37" s="658" t="str">
         <f>IF(O3="No","","Clasificacion AASHTO")</f>
         <v/>
       </c>
-      <c r="G37" s="626"/>
-      <c r="H37" s="629" t="str">
+      <c r="G37" s="658"/>
+      <c r="H37" s="660" t="str">
         <f>IF(O3="No","",Aashto!J26)</f>
         <v/>
       </c>
-      <c r="I37" s="629"/>
+      <c r="I37" s="660"/>
       <c r="J37" s="319"/>
       <c r="K37" s="320"/>
       <c r="L37" s="15"/>
@@ -12636,19 +12602,19 @@
       <c r="A38" s="329">
         <v>200</v>
       </c>
-      <c r="B38" s="621">
+      <c r="B38" s="654">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="C38" s="621"/>
+      <c r="C38" s="654"/>
       <c r="D38" s="330">
         <f t="shared" si="4"/>
         <v>13.456812316430202</v>
       </c>
       <c r="E38" s="313"/>
-      <c r="F38" s="627"/>
-      <c r="G38" s="627"/>
-      <c r="H38" s="630"/>
-      <c r="I38" s="630"/>
+      <c r="F38" s="659"/>
+      <c r="G38" s="659"/>
+      <c r="H38" s="661"/>
+      <c r="I38" s="661"/>
       <c r="J38" s="319"/>
       <c r="K38" s="320"/>
       <c r="L38" s="15"/>
@@ -13540,19 +13506,19 @@
       <c r="Z63" s="51"/>
     </row>
     <row r="64" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="643" t="s">
+      <c r="A64" s="622" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="643"/>
-      <c r="C64" s="643"/>
-      <c r="D64" s="643"/>
-      <c r="E64" s="643"/>
-      <c r="F64" s="643"/>
-      <c r="G64" s="643"/>
-      <c r="H64" s="643"/>
-      <c r="I64" s="643"/>
-      <c r="J64" s="643"/>
-      <c r="K64" s="643"/>
+      <c r="B64" s="622"/>
+      <c r="C64" s="622"/>
+      <c r="D64" s="622"/>
+      <c r="E64" s="622"/>
+      <c r="F64" s="622"/>
+      <c r="G64" s="622"/>
+      <c r="H64" s="622"/>
+      <c r="I64" s="622"/>
+      <c r="J64" s="622"/>
+      <c r="K64" s="622"/>
       <c r="W64" s="51"/>
       <c r="X64" s="51"/>
       <c r="Y64" s="51"/>
@@ -13588,6 +13554,29 @@
     <protectedRange sqref="C10" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="39">
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="T16:V16"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="F35:G36"/>
+    <mergeCell ref="F37:G38"/>
+    <mergeCell ref="H35:I36"/>
+    <mergeCell ref="H37:I38"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C12:H12"/>
     <mergeCell ref="F30:F32"/>
     <mergeCell ref="G30:G32"/>
     <mergeCell ref="A64:K64"/>
@@ -13604,29 +13593,6 @@
     <mergeCell ref="F23:H24"/>
     <mergeCell ref="I23:I24"/>
     <mergeCell ref="F26:I27"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="F35:G36"/>
-    <mergeCell ref="F37:G38"/>
-    <mergeCell ref="H35:I36"/>
-    <mergeCell ref="H37:I38"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -13754,35 +13720,35 @@
       <c r="K7" s="203"/>
     </row>
     <row r="8" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="662" t="s">
+      <c r="A8" s="682" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="662"/>
-      <c r="C8" s="662"/>
-      <c r="D8" s="662"/>
-      <c r="E8" s="662"/>
-      <c r="F8" s="662"/>
-      <c r="G8" s="662"/>
-      <c r="H8" s="662"/>
-      <c r="I8" s="662"/>
-      <c r="J8" s="662"/>
-      <c r="K8" s="662"/>
+      <c r="B8" s="682"/>
+      <c r="C8" s="682"/>
+      <c r="D8" s="682"/>
+      <c r="E8" s="682"/>
+      <c r="F8" s="682"/>
+      <c r="G8" s="682"/>
+      <c r="H8" s="682"/>
+      <c r="I8" s="682"/>
+      <c r="J8" s="682"/>
+      <c r="K8" s="682"/>
     </row>
     <row r="9" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="663">
+      <c r="A9" s="683">
         <f>+K13</f>
         <v>10</v>
       </c>
-      <c r="B9" s="663"/>
-      <c r="C9" s="663"/>
-      <c r="D9" s="663"/>
-      <c r="E9" s="663"/>
-      <c r="F9" s="663"/>
-      <c r="G9" s="663"/>
-      <c r="H9" s="663"/>
-      <c r="I9" s="663"/>
-      <c r="J9" s="663"/>
-      <c r="K9" s="663"/>
+      <c r="B9" s="683"/>
+      <c r="C9" s="683"/>
+      <c r="D9" s="683"/>
+      <c r="E9" s="683"/>
+      <c r="F9" s="683"/>
+      <c r="G9" s="683"/>
+      <c r="H9" s="683"/>
+      <c r="I9" s="683"/>
+      <c r="J9" s="683"/>
+      <c r="K9" s="683"/>
       <c r="O9" s="204"/>
     </row>
     <row r="10" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -13805,14 +13771,14 @@
       <c r="B11" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="664" t="s">
+      <c r="C11" s="684" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="664"/>
-      <c r="E11" s="664"/>
-      <c r="F11" s="664"/>
-      <c r="G11" s="664"/>
-      <c r="H11" s="664"/>
+      <c r="D11" s="684"/>
+      <c r="E11" s="684"/>
+      <c r="F11" s="684"/>
+      <c r="G11" s="684"/>
+      <c r="H11" s="684"/>
       <c r="I11" s="206" t="s">
         <v>38</v>
       </c>
@@ -13833,14 +13799,14 @@
       <c r="B12" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="664" t="s">
+      <c r="C12" s="684" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="664"/>
-      <c r="E12" s="664"/>
-      <c r="F12" s="664"/>
-      <c r="G12" s="664"/>
-      <c r="H12" s="664"/>
+      <c r="D12" s="684"/>
+      <c r="E12" s="684"/>
+      <c r="F12" s="684"/>
+      <c r="G12" s="684"/>
+      <c r="H12" s="684"/>
       <c r="I12" s="39" t="s">
         <v>21</v>
       </c>
@@ -13864,14 +13830,14 @@
       <c r="B13" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="664" t="s">
+      <c r="C13" s="684" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="664"/>
-      <c r="E13" s="664"/>
-      <c r="F13" s="664"/>
-      <c r="G13" s="664"/>
-      <c r="H13" s="664"/>
+      <c r="D13" s="684"/>
+      <c r="E13" s="684"/>
+      <c r="F13" s="684"/>
+      <c r="G13" s="684"/>
+      <c r="H13" s="684"/>
       <c r="I13" s="39" t="s">
         <v>22</v>
       </c>
@@ -13885,8 +13851,8 @@
       <c r="M13" s="209"/>
       <c r="P13" s="212"/>
       <c r="Q13" s="212"/>
-      <c r="R13" s="661"/>
-      <c r="S13" s="661"/>
+      <c r="R13" s="681"/>
+      <c r="S13" s="681"/>
     </row>
     <row r="14" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="34"/>
@@ -13908,19 +13874,19 @@
       <c r="S14" s="217"/>
     </row>
     <row r="15" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="665" t="s">
+      <c r="A15" s="669" t="s">
         <v>229</v>
       </c>
-      <c r="B15" s="666"/>
-      <c r="C15" s="666"/>
-      <c r="D15" s="666"/>
-      <c r="E15" s="666"/>
-      <c r="F15" s="666"/>
-      <c r="G15" s="666"/>
-      <c r="H15" s="666"/>
-      <c r="I15" s="666"/>
-      <c r="J15" s="666"/>
-      <c r="K15" s="667"/>
+      <c r="B15" s="670"/>
+      <c r="C15" s="670"/>
+      <c r="D15" s="670"/>
+      <c r="E15" s="670"/>
+      <c r="F15" s="670"/>
+      <c r="G15" s="670"/>
+      <c r="H15" s="670"/>
+      <c r="I15" s="670"/>
+      <c r="J15" s="670"/>
+      <c r="K15" s="671"/>
       <c r="L15" s="209"/>
       <c r="M15" s="209"/>
       <c r="P15" s="212"/>
@@ -13929,19 +13895,19 @@
       <c r="S15" s="217"/>
     </row>
     <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="668" t="s">
+      <c r="A16" s="672" t="s">
         <v>277</v>
       </c>
-      <c r="B16" s="669"/>
-      <c r="C16" s="669"/>
-      <c r="D16" s="669"/>
-      <c r="E16" s="669"/>
-      <c r="F16" s="669"/>
-      <c r="G16" s="669"/>
-      <c r="H16" s="669"/>
-      <c r="I16" s="669"/>
-      <c r="J16" s="669"/>
-      <c r="K16" s="670"/>
+      <c r="B16" s="673"/>
+      <c r="C16" s="673"/>
+      <c r="D16" s="673"/>
+      <c r="E16" s="673"/>
+      <c r="F16" s="673"/>
+      <c r="G16" s="673"/>
+      <c r="H16" s="673"/>
+      <c r="I16" s="673"/>
+      <c r="J16" s="673"/>
+      <c r="K16" s="674"/>
       <c r="L16" s="209"/>
       <c r="M16" s="209"/>
       <c r="P16" s="212"/>
@@ -13969,19 +13935,19 @@
       <c r="S17" s="217"/>
     </row>
     <row r="18" spans="1:21" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="671" t="s">
+      <c r="A18" s="675" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="636"/>
-      <c r="C18" s="636"/>
-      <c r="D18" s="636"/>
-      <c r="E18" s="636"/>
-      <c r="F18" s="636"/>
-      <c r="G18" s="636"/>
-      <c r="H18" s="636"/>
-      <c r="I18" s="636"/>
-      <c r="J18" s="636"/>
-      <c r="K18" s="637"/>
+      <c r="B18" s="645"/>
+      <c r="C18" s="645"/>
+      <c r="D18" s="645"/>
+      <c r="E18" s="645"/>
+      <c r="F18" s="645"/>
+      <c r="G18" s="645"/>
+      <c r="H18" s="645"/>
+      <c r="I18" s="645"/>
+      <c r="J18" s="645"/>
+      <c r="K18" s="646"/>
       <c r="M18" s="209"/>
       <c r="P18" s="212"/>
       <c r="Q18" s="212"/>
@@ -14098,8 +14064,8 @@
     </row>
     <row r="23" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="231"/>
-      <c r="I23" s="672"/>
-      <c r="J23" s="672"/>
+      <c r="I23" s="676"/>
+      <c r="J23" s="676"/>
       <c r="K23" s="232"/>
       <c r="L23" s="209"/>
       <c r="M23" s="233"/>
@@ -14107,41 +14073,41 @@
     </row>
     <row r="24" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="235"/>
-      <c r="D24" s="673" t="s">
+      <c r="D24" s="677" t="s">
         <v>232</v>
       </c>
-      <c r="E24" s="674"/>
-      <c r="F24" s="674"/>
-      <c r="G24" s="675" t="s">
+      <c r="E24" s="678"/>
+      <c r="F24" s="678"/>
+      <c r="G24" s="679" t="s">
         <v>233</v>
       </c>
-      <c r="H24" s="676"/>
-      <c r="I24" s="677"/>
-      <c r="J24" s="677"/>
+      <c r="H24" s="680"/>
+      <c r="I24" s="667"/>
+      <c r="J24" s="667"/>
       <c r="K24" s="236"/>
       <c r="L24" s="209"/>
       <c r="M24" s="237"/>
-      <c r="O24" s="678" t="s">
+      <c r="O24" s="662" t="s">
         <v>232</v>
       </c>
-      <c r="P24" s="679"/>
+      <c r="P24" s="663"/>
       <c r="Q24" s="238" t="s">
         <v>231</v>
       </c>
-      <c r="R24" s="678" t="s">
+      <c r="R24" s="662" t="s">
         <v>233</v>
       </c>
-      <c r="S24" s="680"/>
+      <c r="S24" s="664"/>
       <c r="T24" s="238" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="235"/>
-      <c r="B25" s="681" t="s">
+      <c r="B25" s="665" t="s">
         <v>234</v>
       </c>
-      <c r="C25" s="682"/>
+      <c r="C25" s="666"/>
       <c r="D25" s="239" t="str">
         <f>IF($Q$24="NO","",O25)</f>
         <v/>
@@ -14162,8 +14128,8 @@
         <f>IF($T$24="NO","",S25)</f>
         <v/>
       </c>
-      <c r="I25" s="677"/>
-      <c r="J25" s="677"/>
+      <c r="I25" s="667"/>
+      <c r="J25" s="667"/>
       <c r="K25" s="236"/>
       <c r="L25" s="209"/>
       <c r="M25" s="237"/>
@@ -14212,8 +14178,8 @@
         <f>IF($T$24="NO","",S26)</f>
         <v/>
       </c>
-      <c r="I26" s="683"/>
-      <c r="J26" s="683"/>
+      <c r="I26" s="668"/>
+      <c r="J26" s="668"/>
       <c r="K26" s="249"/>
       <c r="L26" s="250"/>
       <c r="M26" s="237"/>
@@ -14928,19 +14894,19 @@
     </row>
     <row r="49" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="643" t="s">
+      <c r="A50" s="622" t="s">
         <v>41</v>
       </c>
-      <c r="B50" s="643"/>
-      <c r="C50" s="643"/>
-      <c r="D50" s="643"/>
-      <c r="E50" s="643"/>
-      <c r="F50" s="643"/>
-      <c r="G50" s="643"/>
-      <c r="H50" s="643"/>
-      <c r="I50" s="643"/>
-      <c r="J50" s="643"/>
-      <c r="K50" s="643"/>
+      <c r="B50" s="622"/>
+      <c r="C50" s="622"/>
+      <c r="D50" s="622"/>
+      <c r="E50" s="622"/>
+      <c r="F50" s="622"/>
+      <c r="G50" s="622"/>
+      <c r="H50" s="622"/>
+      <c r="I50" s="622"/>
+      <c r="J50" s="622"/>
+      <c r="K50" s="622"/>
     </row>
     <row r="51" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="52" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -14950,11 +14916,12 @@
     <protectedRange sqref="C11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="19">
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
     <mergeCell ref="A50:K50"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A16:K16"/>
@@ -14963,12 +14930,11 @@
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="I24:J24"/>
-    <mergeCell ref="R13:S13"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="A9:K9"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q24 T24" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -15082,33 +15048,33 @@
       <c r="J7" s="203"/>
     </row>
     <row r="8" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="662" t="s">
+      <c r="A8" s="682" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="662"/>
-      <c r="C8" s="662"/>
-      <c r="D8" s="662"/>
-      <c r="E8" s="662"/>
-      <c r="F8" s="662"/>
-      <c r="G8" s="662"/>
-      <c r="H8" s="662"/>
-      <c r="I8" s="662"/>
-      <c r="J8" s="662"/>
+      <c r="B8" s="682"/>
+      <c r="C8" s="682"/>
+      <c r="D8" s="682"/>
+      <c r="E8" s="682"/>
+      <c r="F8" s="682"/>
+      <c r="G8" s="682"/>
+      <c r="H8" s="682"/>
+      <c r="I8" s="682"/>
+      <c r="J8" s="682"/>
     </row>
     <row r="9" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="690">
+      <c r="A9" s="685">
         <f>J13</f>
         <v>1</v>
       </c>
-      <c r="B9" s="690"/>
-      <c r="C9" s="690"/>
-      <c r="D9" s="690"/>
-      <c r="E9" s="690"/>
-      <c r="F9" s="690"/>
-      <c r="G9" s="690"/>
-      <c r="H9" s="690"/>
-      <c r="I9" s="690"/>
-      <c r="J9" s="690"/>
+      <c r="B9" s="685"/>
+      <c r="C9" s="685"/>
+      <c r="D9" s="685"/>
+      <c r="E9" s="685"/>
+      <c r="F9" s="685"/>
+      <c r="G9" s="685"/>
+      <c r="H9" s="685"/>
+      <c r="I9" s="685"/>
+      <c r="J9" s="685"/>
       <c r="O9" s="204"/>
     </row>
     <row r="10" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -15130,13 +15096,13 @@
       <c r="B11" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="664" t="s">
+      <c r="C11" s="684" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="664"/>
-      <c r="E11" s="664"/>
-      <c r="F11" s="664"/>
-      <c r="G11" s="664"/>
+      <c r="D11" s="684"/>
+      <c r="E11" s="684"/>
+      <c r="F11" s="684"/>
+      <c r="G11" s="684"/>
       <c r="H11" s="206" t="s">
         <v>38</v>
       </c>
@@ -15158,13 +15124,13 @@
       <c r="B12" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="664" t="s">
+      <c r="C12" s="684" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="664"/>
-      <c r="E12" s="664"/>
-      <c r="F12" s="664"/>
-      <c r="G12" s="664"/>
+      <c r="D12" s="684"/>
+      <c r="E12" s="684"/>
+      <c r="F12" s="684"/>
+      <c r="G12" s="684"/>
       <c r="H12" s="39" t="s">
         <v>21</v>
       </c>
@@ -15188,13 +15154,13 @@
       <c r="B13" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="664" t="s">
+      <c r="C13" s="684" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="664"/>
-      <c r="E13" s="664"/>
-      <c r="F13" s="664"/>
-      <c r="G13" s="664"/>
+      <c r="D13" s="684"/>
+      <c r="E13" s="684"/>
+      <c r="F13" s="684"/>
+      <c r="G13" s="684"/>
       <c r="H13" s="39" t="s">
         <v>22</v>
       </c>
@@ -15207,8 +15173,8 @@
       <c r="K13" s="209"/>
       <c r="L13" s="209"/>
       <c r="M13" s="209"/>
-      <c r="P13" s="661"/>
-      <c r="Q13" s="661"/>
+      <c r="P13" s="681"/>
+      <c r="Q13" s="681"/>
     </row>
     <row r="14" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="34"/>
@@ -15228,34 +15194,34 @@
       <c r="Q14" s="217"/>
     </row>
     <row r="15" spans="1:17" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="665" t="s">
+      <c r="A15" s="669" t="s">
         <v>259</v>
       </c>
-      <c r="B15" s="666"/>
-      <c r="C15" s="666"/>
-      <c r="D15" s="666"/>
-      <c r="E15" s="666"/>
-      <c r="F15" s="666"/>
-      <c r="G15" s="666"/>
-      <c r="H15" s="666"/>
-      <c r="I15" s="666"/>
-      <c r="J15" s="667"/>
+      <c r="B15" s="670"/>
+      <c r="C15" s="670"/>
+      <c r="D15" s="670"/>
+      <c r="E15" s="670"/>
+      <c r="F15" s="670"/>
+      <c r="G15" s="670"/>
+      <c r="H15" s="670"/>
+      <c r="I15" s="670"/>
+      <c r="J15" s="671"/>
       <c r="K15" s="209"/>
       <c r="L15" s="209"/>
     </row>
     <row r="16" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="668" t="s">
+      <c r="A16" s="672" t="s">
         <v>260</v>
       </c>
-      <c r="B16" s="684"/>
-      <c r="C16" s="684"/>
-      <c r="D16" s="684"/>
-      <c r="E16" s="684"/>
-      <c r="F16" s="684"/>
-      <c r="G16" s="684"/>
-      <c r="H16" s="684"/>
-      <c r="I16" s="684"/>
-      <c r="J16" s="685"/>
+      <c r="B16" s="686"/>
+      <c r="C16" s="686"/>
+      <c r="D16" s="686"/>
+      <c r="E16" s="686"/>
+      <c r="F16" s="686"/>
+      <c r="G16" s="686"/>
+      <c r="H16" s="686"/>
+      <c r="I16" s="686"/>
+      <c r="J16" s="687"/>
       <c r="K16" s="209"/>
       <c r="L16" s="209"/>
     </row>
@@ -15274,18 +15240,18 @@
       <c r="L17" s="209"/>
     </row>
     <row r="18" spans="1:18" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="636" t="s">
+      <c r="A18" s="645" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="636"/>
-      <c r="C18" s="636"/>
-      <c r="D18" s="636"/>
-      <c r="E18" s="636"/>
-      <c r="F18" s="636"/>
-      <c r="G18" s="636"/>
-      <c r="H18" s="636"/>
-      <c r="I18" s="636"/>
-      <c r="J18" s="636"/>
+      <c r="B18" s="645"/>
+      <c r="C18" s="645"/>
+      <c r="D18" s="645"/>
+      <c r="E18" s="645"/>
+      <c r="F18" s="645"/>
+      <c r="G18" s="645"/>
+      <c r="H18" s="645"/>
+      <c r="I18" s="645"/>
+      <c r="J18" s="645"/>
       <c r="L18" s="209"/>
     </row>
     <row r="19" spans="1:18" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -15400,12 +15366,12 @@
     <row r="24" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="402"/>
       <c r="B24" s="400"/>
-      <c r="C24" s="686" t="s">
+      <c r="C24" s="688" t="s">
         <v>261</v>
       </c>
-      <c r="D24" s="687"/>
-      <c r="E24" s="687"/>
-      <c r="F24" s="688"/>
+      <c r="D24" s="689"/>
+      <c r="E24" s="689"/>
+      <c r="F24" s="690"/>
       <c r="G24" s="400"/>
       <c r="H24" s="400"/>
       <c r="I24" s="400"/>
@@ -15522,10 +15488,10 @@
     <row r="28" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="402"/>
       <c r="B28" s="282"/>
-      <c r="C28" s="689"/>
-      <c r="D28" s="689"/>
-      <c r="E28" s="689"/>
-      <c r="F28" s="689"/>
+      <c r="C28" s="691"/>
+      <c r="D28" s="691"/>
+      <c r="E28" s="691"/>
+      <c r="F28" s="691"/>
       <c r="G28" s="396"/>
       <c r="H28" s="411"/>
       <c r="I28" s="411"/>
@@ -15549,12 +15515,12 @@
     <row r="29" spans="1:18" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="402"/>
       <c r="B29" s="282"/>
-      <c r="C29" s="686" t="s">
+      <c r="C29" s="688" t="s">
         <v>267</v>
       </c>
-      <c r="D29" s="687"/>
-      <c r="E29" s="687"/>
-      <c r="F29" s="688"/>
+      <c r="D29" s="689"/>
+      <c r="E29" s="689"/>
+      <c r="F29" s="690"/>
       <c r="G29" s="426" t="s">
         <v>268</v>
       </c>
@@ -15983,18 +15949,18 @@
     </row>
     <row r="53" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="643" t="s">
+      <c r="A54" s="622" t="s">
         <v>41</v>
       </c>
-      <c r="B54" s="643"/>
-      <c r="C54" s="643"/>
-      <c r="D54" s="643"/>
-      <c r="E54" s="643"/>
-      <c r="F54" s="643"/>
-      <c r="G54" s="643"/>
-      <c r="H54" s="643"/>
-      <c r="I54" s="643"/>
-      <c r="J54" s="643"/>
+      <c r="B54" s="622"/>
+      <c r="C54" s="622"/>
+      <c r="D54" s="622"/>
+      <c r="E54" s="622"/>
+      <c r="F54" s="622"/>
+      <c r="G54" s="622"/>
+      <c r="H54" s="622"/>
+      <c r="I54" s="622"/>
+      <c r="J54" s="622"/>
     </row>
     <row r="55" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16004,12 +15970,6 @@
     <protectedRange sqref="C11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="13">
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
     <mergeCell ref="A54:J54"/>
     <mergeCell ref="A15:J15"/>
     <mergeCell ref="A16:J16"/>
@@ -16017,6 +15977,12 @@
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="C29:F29"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -16048,15 +16014,15 @@
       <c r="A1" s="145" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="691" t="s">
+      <c r="B1" s="709" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="691"/>
-      <c r="D1" s="691"/>
-      <c r="E1" s="691"/>
-      <c r="F1" s="691"/>
-      <c r="G1" s="691"/>
-      <c r="H1" s="691"/>
+      <c r="C1" s="709"/>
+      <c r="D1" s="709"/>
+      <c r="E1" s="709"/>
+      <c r="F1" s="709"/>
+      <c r="G1" s="709"/>
+      <c r="H1" s="709"/>
       <c r="I1" s="145"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -16194,29 +16160,29 @@
     </row>
     <row r="8" spans="1:17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="145"/>
-      <c r="B8" s="692" t="s">
+      <c r="B8" s="710" t="s">
         <v>168</v>
       </c>
-      <c r="C8" s="692"/>
-      <c r="D8" s="692"/>
+      <c r="C8" s="710"/>
+      <c r="D8" s="710"/>
       <c r="E8" s="154" t="s">
         <v>169</v>
       </c>
       <c r="F8" s="155" t="s">
         <v>170</v>
       </c>
-      <c r="G8" s="693" t="s">
+      <c r="G8" s="711" t="s">
         <v>171</v>
       </c>
-      <c r="H8" s="693"/>
+      <c r="H8" s="711"/>
       <c r="I8" s="145"/>
       <c r="L8" s="156" t="s">
         <v>172</v>
       </c>
-      <c r="M8" s="694" t="s">
+      <c r="M8" s="712" t="s">
         <v>173</v>
       </c>
-      <c r="N8" s="694"/>
+      <c r="N8" s="712"/>
       <c r="O8" s="157" t="s">
         <v>174</v>
       </c>
@@ -16229,13 +16195,13 @@
     </row>
     <row r="9" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="145"/>
-      <c r="B9" s="695" t="s">
+      <c r="B9" s="713" t="s">
         <v>177</v>
       </c>
-      <c r="C9" s="697" t="s">
+      <c r="C9" s="715" t="s">
         <v>178</v>
       </c>
-      <c r="D9" s="699" t="s">
+      <c r="D9" s="717" t="s">
         <v>179</v>
       </c>
       <c r="E9" s="159" t="s">
@@ -16244,10 +16210,10 @@
       <c r="F9" s="160" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="700" t="s">
+      <c r="G9" s="718" t="s">
         <v>182</v>
       </c>
-      <c r="H9" s="701"/>
+      <c r="H9" s="719"/>
       <c r="I9" s="145"/>
       <c r="L9" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&lt;5,CU&gt;=4,CC&gt;=1,CC&lt;=3),"GW","")</f>
@@ -16276,19 +16242,19 @@
     </row>
     <row r="10" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="145"/>
-      <c r="B10" s="695"/>
-      <c r="C10" s="697"/>
-      <c r="D10" s="699"/>
+      <c r="B10" s="713"/>
+      <c r="C10" s="715"/>
+      <c r="D10" s="717"/>
       <c r="E10" s="161" t="s">
         <v>183</v>
       </c>
       <c r="F10" s="162" t="s">
         <v>184</v>
       </c>
-      <c r="G10" s="702" t="s">
+      <c r="G10" s="720" t="s">
         <v>185</v>
       </c>
-      <c r="H10" s="703"/>
+      <c r="H10" s="721"/>
       <c r="I10" s="145"/>
       <c r="L10" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&lt;5,OR(CU&lt;4,CC&lt;1,CC&gt;3)),"GP","")</f>
@@ -16313,9 +16279,9 @@
     </row>
     <row r="11" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="145"/>
-      <c r="B11" s="695"/>
-      <c r="C11" s="697"/>
-      <c r="D11" s="699" t="s">
+      <c r="B11" s="713"/>
+      <c r="C11" s="715"/>
+      <c r="D11" s="717" t="s">
         <v>186</v>
       </c>
       <c r="E11" s="161" t="s">
@@ -16327,7 +16293,7 @@
       <c r="G11" s="164" t="s">
         <v>189</v>
       </c>
-      <c r="H11" s="704" t="s">
+      <c r="H11" s="722" t="s">
         <v>190</v>
       </c>
       <c r="I11" s="145"/>
@@ -16346,9 +16312,9 @@
     </row>
     <row r="12" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="145"/>
-      <c r="B12" s="695"/>
-      <c r="C12" s="698"/>
-      <c r="D12" s="699"/>
+      <c r="B12" s="713"/>
+      <c r="C12" s="716"/>
+      <c r="D12" s="717"/>
       <c r="E12" s="165" t="s">
         <v>191</v>
       </c>
@@ -16358,7 +16324,7 @@
       <c r="G12" s="164" t="s">
         <v>193</v>
       </c>
-      <c r="H12" s="705"/>
+      <c r="H12" s="723"/>
       <c r="I12" s="145"/>
       <c r="L12" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&gt;=0.5*(100-N_200),N_200&gt;=12,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"GC","")</f>
@@ -16371,11 +16337,11 @@
     </row>
     <row r="13" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="145"/>
-      <c r="B13" s="695"/>
-      <c r="C13" s="697" t="s">
+      <c r="B13" s="713"/>
+      <c r="C13" s="715" t="s">
         <v>194</v>
       </c>
-      <c r="D13" s="699" t="s">
+      <c r="D13" s="717" t="s">
         <v>195</v>
       </c>
       <c r="E13" s="166" t="s">
@@ -16384,10 +16350,10 @@
       <c r="F13" s="167" t="s">
         <v>197</v>
       </c>
-      <c r="G13" s="706" t="s">
+      <c r="G13" s="724" t="s">
         <v>198</v>
       </c>
-      <c r="H13" s="707"/>
+      <c r="H13" s="725"/>
       <c r="I13" s="145"/>
       <c r="L13" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&lt;5,CU&gt;=6,CC&gt;=1,CC&lt;=3),"SW","")</f>
@@ -16412,19 +16378,19 @@
     </row>
     <row r="14" spans="1:17" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="145"/>
-      <c r="B14" s="695"/>
-      <c r="C14" s="697"/>
-      <c r="D14" s="699"/>
+      <c r="B14" s="713"/>
+      <c r="C14" s="715"/>
+      <c r="D14" s="717"/>
       <c r="E14" s="166" t="s">
         <v>199</v>
       </c>
       <c r="F14" s="167" t="s">
         <v>200</v>
       </c>
-      <c r="G14" s="706" t="s">
+      <c r="G14" s="724" t="s">
         <v>201</v>
       </c>
-      <c r="H14" s="707"/>
+      <c r="H14" s="725"/>
       <c r="I14" s="145"/>
       <c r="L14" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&lt;5,OR(CU&lt;6,CC&lt;1,CC&gt;3)),"SP","")</f>
@@ -16449,9 +16415,9 @@
     </row>
     <row r="15" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="145"/>
-      <c r="B15" s="695"/>
-      <c r="C15" s="697"/>
-      <c r="D15" s="699" t="s">
+      <c r="B15" s="713"/>
+      <c r="C15" s="715"/>
+      <c r="D15" s="717" t="s">
         <v>202</v>
       </c>
       <c r="E15" s="166" t="s">
@@ -16463,7 +16429,7 @@
       <c r="G15" s="169" t="s">
         <v>205</v>
       </c>
-      <c r="H15" s="708" t="s">
+      <c r="H15" s="692" t="s">
         <v>206</v>
       </c>
       <c r="I15" s="145"/>
@@ -16482,9 +16448,9 @@
     </row>
     <row r="16" spans="1:17" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="145"/>
-      <c r="B16" s="696"/>
-      <c r="C16" s="697"/>
-      <c r="D16" s="699"/>
+      <c r="B16" s="714"/>
+      <c r="C16" s="715"/>
+      <c r="D16" s="717"/>
       <c r="E16" s="170" t="s">
         <v>207</v>
       </c>
@@ -16494,7 +16460,7 @@
       <c r="G16" s="167" t="s">
         <v>209</v>
       </c>
-      <c r="H16" s="709"/>
+      <c r="H16" s="693"/>
       <c r="I16" s="145"/>
       <c r="L16" s="140" t="str">
         <f>IF(AND(N_200&lt;50,(100-N_40)&lt;0.5*(100-N_200),N_200&gt;=12,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"SC","")</f>
@@ -16507,23 +16473,23 @@
     </row>
     <row r="17" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="145"/>
-      <c r="B17" s="710" t="s">
+      <c r="B17" s="694" t="s">
         <v>210</v>
       </c>
-      <c r="C17" s="713" t="s">
+      <c r="C17" s="697" t="s">
         <v>211</v>
       </c>
-      <c r="D17" s="714"/>
+      <c r="D17" s="698"/>
       <c r="E17" s="171" t="s">
         <v>212</v>
       </c>
       <c r="F17" s="172" t="s">
         <v>213</v>
       </c>
-      <c r="G17" s="719" t="s">
+      <c r="G17" s="703" t="s">
         <v>214</v>
       </c>
-      <c r="H17" s="720"/>
+      <c r="H17" s="704"/>
       <c r="I17" s="145"/>
       <c r="L17" s="140" t="str">
         <f>IF(AND(OR(L2="Inorganico"),N_200&gt;=50,Ll&lt;50,OR(IP&lt;4,AND(IP&lt;0.73*(Ll-20)))),"ML","")</f>
@@ -16536,17 +16502,17 @@
     </row>
     <row r="18" spans="1:16" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="145"/>
-      <c r="B18" s="711"/>
-      <c r="C18" s="715"/>
-      <c r="D18" s="716"/>
+      <c r="B18" s="695"/>
+      <c r="C18" s="699"/>
+      <c r="D18" s="700"/>
       <c r="E18" s="171" t="s">
         <v>215</v>
       </c>
       <c r="F18" s="172" t="s">
         <v>216</v>
       </c>
-      <c r="G18" s="721"/>
-      <c r="H18" s="722"/>
+      <c r="G18" s="705"/>
+      <c r="H18" s="706"/>
       <c r="I18" s="145"/>
       <c r="L18" s="140" t="str">
         <f>IF(AND(OR(L2="Inorganico"),N_200&gt;=50,Ll&lt;50,IP&gt;=7,IP&gt;=0.73*(Ll-20)),"CL","")</f>
@@ -16559,9 +16525,9 @@
     </row>
     <row r="19" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="145"/>
-      <c r="B19" s="711"/>
-      <c r="C19" s="717"/>
-      <c r="D19" s="718"/>
+      <c r="B19" s="695"/>
+      <c r="C19" s="701"/>
+      <c r="D19" s="702"/>
       <c r="E19" s="171" t="s">
         <v>217</v>
       </c>
@@ -16582,11 +16548,11 @@
     </row>
     <row r="20" spans="1:16" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="145"/>
-      <c r="B20" s="711"/>
-      <c r="C20" s="715" t="s">
+      <c r="B20" s="695"/>
+      <c r="C20" s="699" t="s">
         <v>219</v>
       </c>
-      <c r="D20" s="723"/>
+      <c r="D20" s="707"/>
       <c r="E20" s="175" t="s">
         <v>220</v>
       </c>
@@ -16607,9 +16573,9 @@
     </row>
     <row r="21" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="145"/>
-      <c r="B21" s="711"/>
-      <c r="C21" s="715"/>
-      <c r="D21" s="723"/>
+      <c r="B21" s="695"/>
+      <c r="C21" s="699"/>
+      <c r="D21" s="707"/>
       <c r="E21" s="175" t="s">
         <v>222</v>
       </c>
@@ -16630,9 +16596,9 @@
     </row>
     <row r="22" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="145"/>
-      <c r="B22" s="711"/>
-      <c r="C22" s="717"/>
-      <c r="D22" s="724"/>
+      <c r="B22" s="695"/>
+      <c r="C22" s="701"/>
+      <c r="D22" s="708"/>
       <c r="E22" s="177" t="s">
         <v>224</v>
       </c>
@@ -16653,11 +16619,11 @@
     </row>
     <row r="23" spans="1:16" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="145"/>
-      <c r="B23" s="711"/>
-      <c r="C23" s="713" t="s">
+      <c r="B23" s="695"/>
+      <c r="C23" s="697" t="s">
         <v>226</v>
       </c>
-      <c r="D23" s="714"/>
+      <c r="D23" s="698"/>
       <c r="E23" s="178" t="s">
         <v>227</v>
       </c>
@@ -16678,7 +16644,7 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="145"/>
-      <c r="B24" s="712"/>
+      <c r="B24" s="696"/>
       <c r="C24" s="180"/>
       <c r="D24" s="181"/>
       <c r="E24" s="182"/>
@@ -16785,12 +16751,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="B17:B24"/>
-    <mergeCell ref="C17:D19"/>
-    <mergeCell ref="G17:H18"/>
-    <mergeCell ref="C20:D22"/>
-    <mergeCell ref="C23:D23"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="G8:H8"/>
@@ -16807,6 +16767,12 @@
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="D15:D16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="B17:B24"/>
+    <mergeCell ref="C17:D19"/>
+    <mergeCell ref="G17:H18"/>
+    <mergeCell ref="C20:D22"/>
+    <mergeCell ref="C23:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -16882,71 +16848,71 @@
     </row>
     <row r="4" spans="1:16" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="72"/>
-      <c r="B4" s="731" t="s">
+      <c r="B4" s="732" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="732"/>
-      <c r="D4" s="733" t="s">
+      <c r="C4" s="733"/>
+      <c r="D4" s="734" t="s">
         <v>101</v>
       </c>
-      <c r="E4" s="733"/>
-      <c r="F4" s="733"/>
-      <c r="G4" s="733"/>
-      <c r="H4" s="733"/>
-      <c r="I4" s="733"/>
-      <c r="J4" s="733"/>
-      <c r="K4" s="734" t="s">
+      <c r="E4" s="734"/>
+      <c r="F4" s="734"/>
+      <c r="G4" s="734"/>
+      <c r="H4" s="734"/>
+      <c r="I4" s="734"/>
+      <c r="J4" s="734"/>
+      <c r="K4" s="735" t="s">
         <v>102</v>
       </c>
-      <c r="L4" s="735"/>
-      <c r="M4" s="735"/>
-      <c r="N4" s="735"/>
-      <c r="O4" s="736"/>
+      <c r="L4" s="736"/>
+      <c r="M4" s="736"/>
+      <c r="N4" s="736"/>
+      <c r="O4" s="737"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="72"/>
-      <c r="B5" s="737" t="s">
+      <c r="B5" s="738" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="738"/>
-      <c r="D5" s="741" t="s">
+      <c r="C5" s="739"/>
+      <c r="D5" s="742" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="742"/>
-      <c r="F5" s="743" t="s">
+      <c r="E5" s="743"/>
+      <c r="F5" s="744" t="s">
         <v>105</v>
       </c>
-      <c r="G5" s="741" t="s">
+      <c r="G5" s="742" t="s">
         <v>106</v>
       </c>
-      <c r="H5" s="745"/>
-      <c r="I5" s="745"/>
-      <c r="J5" s="742"/>
-      <c r="K5" s="746" t="s">
+      <c r="H5" s="746"/>
+      <c r="I5" s="746"/>
+      <c r="J5" s="743"/>
+      <c r="K5" s="747" t="s">
         <v>107</v>
       </c>
-      <c r="L5" s="748" t="s">
+      <c r="L5" s="749" t="s">
         <v>108</v>
       </c>
-      <c r="M5" s="750" t="s">
+      <c r="M5" s="751" t="s">
         <v>109</v>
       </c>
-      <c r="N5" s="752" t="s">
+      <c r="N5" s="753" t="s">
         <v>110</v>
       </c>
-      <c r="O5" s="753"/>
+      <c r="O5" s="754"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="72"/>
-      <c r="B6" s="739"/>
-      <c r="C6" s="740"/>
+      <c r="B6" s="740"/>
+      <c r="C6" s="741"/>
       <c r="D6" s="76" t="s">
         <v>111</v>
       </c>
       <c r="E6" s="77" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="744"/>
+      <c r="F6" s="745"/>
       <c r="G6" s="76" t="s">
         <v>113</v>
       </c>
@@ -16959,9 +16925,9 @@
       <c r="J6" s="77" t="s">
         <v>116</v>
       </c>
-      <c r="K6" s="747"/>
-      <c r="L6" s="749"/>
-      <c r="M6" s="751"/>
+      <c r="K6" s="748"/>
+      <c r="L6" s="750"/>
+      <c r="M6" s="752"/>
       <c r="N6" s="80" t="s">
         <v>117</v>
       </c>
@@ -17361,21 +17327,21 @@
         <f>+D38</f>
         <v>0</v>
       </c>
-      <c r="D23" s="725">
+      <c r="D23" s="726">
         <v>0</v>
       </c>
-      <c r="E23" s="726"/>
+      <c r="E23" s="727"/>
       <c r="F23" s="133">
         <v>0</v>
       </c>
-      <c r="G23" s="725">
+      <c r="G23" s="726">
         <v>0</v>
       </c>
-      <c r="H23" s="727"/>
-      <c r="I23" s="728" t="s">
+      <c r="H23" s="728"/>
+      <c r="I23" s="729" t="s">
         <v>145</v>
       </c>
-      <c r="J23" s="726"/>
+      <c r="J23" s="727"/>
       <c r="K23" s="134" t="s">
         <v>146</v>
       </c>
@@ -17438,11 +17404,11 @@
       <c r="G26" s="139"/>
       <c r="H26" s="74"/>
       <c r="I26" s="74"/>
-      <c r="J26" s="729" t="str">
+      <c r="J26" s="730" t="str">
         <f>+D31&amp;" "&amp;F38</f>
         <v>A-1-a (0)</v>
       </c>
-      <c r="K26" s="730"/>
+      <c r="K26" s="731"/>
       <c r="L26" s="72"/>
       <c r="M26" s="72"/>
       <c r="N26" s="72"/>
@@ -17702,10 +17668,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="754" t="s">
+      <c r="A2" s="755" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="754"/>
+      <c r="B2" s="755"/>
       <c r="C2" s="6" t="s">
         <v>11</v>
       </c>

</xml_diff>